<commit_message>
docs: add Epic 8 (Backend Optimization) tracker + Sprint 1 analysis + program dashboard
- Epic 8 tracker (Cover + Dashboard): 10 sprint headers for the backend
  modularization / SaaS-ready FastAPI restructure. Sprint plan only, no task
  backlog yet (filled per sprint as picked up).
- Sprint 1 backend current-state analysis: server.py is a 6,665-line monolith
  (86 inline endpoints, 35 models, ~900-line _bootstrap); core.py is a 775-line
  kitchen sink. Documents the target domain-modular architecture + strangler-fig
  migration order. For sign-off before any code moves.
- Master Tracker: add Epic 8 row after Epic 7.
- Build Ledger: warm, responsive HTML dashboard over all 7 epics -> 59 sprints ->
  371 tasks with epic/sprint/task drill-down, light+dark themes, and mobile parity.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -589,6 +589,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -825,48 +826,73 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Epic 8</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Backend Optimization &amp; Modularization (10 sprints; finishes the Phase A/B migration; Sprint 1 = modular foundation + backend analysis)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>DecisionOS_Epic8_Backend_Optimization.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Testing Plan</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Automated + Alpha + Beta + GA</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>See Epic 1 Testing Plan sheet</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Go-Live</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Go-Live Checklist</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Final SaaS-scale readiness</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>See Epic 1 Go-Live Checklist sheet</t>
         </is>

</xml_diff>

<commit_message>
Add Epic 9 -- Landing Page tracker
- docs/DecisionOS_Epic9_Landing_Page.xlsx: 8 sprints, 59 tasks, 55 done
  (93%). Cover / Dashboard / Backlog sheets, styling cloned from Epic 8
  so the format matches. Sprints 1-7 are retrospective (the landing page
  shipped in one continuous build over ~4 days); Sprint 8 tracks the
  four open items (FAQ direction, logo colour mismatch, GitHub Pages
  hosting, post-Pages production deployment).
- docs/DecisionOS_Master_Tracker.xlsx: Epic 9 row appended after Epic 8;
  all-epics rollup recomputed to 319/442 (72%). Merges cleanly with the
  upstream Epic 8 S2 update (15/16, 94%). No existing epic rows changed.
- landing-page/landing-page-build-tracker.md: source content the tracker
  is populated from (retrospective build log). Referenced in the
  Backlog Source column.
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -585,7 +585,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>All-epics progress: 264 of 383 items resolved  (69%)</t>
+          <t>All-epics progress: 319 of 442 items resolved  (72%)</t>
         </is>
       </c>
     </row>
@@ -859,48 +859,81 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Epic 9</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Landing Page (marketing site -- hero, problem, product tour, ICP, pricing, CEO Brief teaser, final CTA)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>DecisionOS_Epic9_Landing_Page.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Testing Plan</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Automated + Alpha + Beta + GA</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>See Epic 1 Testing Plan sheet</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Go-Live</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Go-Live Checklist</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Final SaaS-scale readiness</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>See Epic 1 Go-Live Checklist sheet</t>
         </is>

</xml_diff>

<commit_message>
Epic 10: Admin / Platform Console tracker (Sprint 0 shipped + S1-S10 plan)
New epic for the platform super-admin / support console. Audited what already
ships and recorded it as Sprint 0 (10/10 Done): separate /admin auth
(dos_admin_token, lockout, immutable platform_audit), 24 API routes in
routers/admin.py, and an 8-tab portal (Overview, Usage, AI Keys, Workspaces,
Users, Maintenance, Audit Log, Health -- pages/admin/, 947 lines).

Forward sprints S1-S10 laid out at scope level (all four founder-prioritized
areas): S1 Tenant 360 & cross-tenant search, S2 Support impersonation
(view-as-tenant), S3 Support desk & tickets, S4 Billing & subscriptions
(Razorpay), S5 Observability & logs, S6 Feature flags, S7 Admin RBAC & 2FA,
S8 Announcements/comms, S9 DPDP/GDPR data ops, S10 polish/tests.

Registered in Master (Epic 10 = 10/71; program 375/559) and rebuilt the
program dashboard HTML.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -585,7 +585,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>All-epics progress: 365 of 488 items resolved  (75%)</t>
+          <t>All-epics progress: 375 of 559 items resolved  (67%)</t>
         </is>
       </c>
     </row>
@@ -891,48 +891,81 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Epic 10</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Admin / Platform Console (super-admin console: tenant 360, impersonation, support desk, billing, observability; Sprint 0 = shipped)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>DecisionOS_Epic10_Admin_Console.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Testing Plan</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Automated + Alpha + Beta + GA</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>See Epic 1 Testing Plan sheet</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Go-Live</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Go-Live Checklist</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Final SaaS-scale readiness</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>See Epic 1 Go-Live Checklist sheet</t>
         </is>

</xml_diff>

<commit_message>
docs: bump Master Tracker + ledger for U10-QA.1
Discovered while browsing the ledger — Sprint 0 correctly showed 11/11
after the QA fix landed, but the Epic 10 top-tile still read 61/73 (from
the Master Tracker overview row, which I forgot to bump alongside the
Epic 10 xlsx in 128ce99). Master Tracker Epic 10 -> 62/74; all-epics
banner 452/605 -> 453/606. Dashboard HTML regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -585,7 +585,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>All-epics progress: 452 of 605 items resolved  (65%)</t>
+          <t>All-epics progress: 453 of 606 items resolved  (65%)</t>
         </is>
       </c>
     </row>
@@ -903,14 +903,14 @@
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>83%</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">

</xml_diff>

<commit_message>
docs(ledger): mark Epic 3 + Epic 10 Done across ledger + Master Tracker
The epic cards read their badge from the epic-detail `status` field, which was
still "In Progress" for Epic 3 and Epic 10 even though both are at 100%. Set both
to Done in the ledger (master.epics + epic detail) and in the authoritative
Master Tracker (Overview Dashboard), so the badges, the "epics complete" counter
(now 6 of 10), and any future ledger rebuild all agree:

  - Epic 3 (AI Foundation): 38/38, 100%, Done (active scope; 5 items future-scoped
    + 7 moved to Epic 6, noted in the epic theme/backlog).
  - Epic 10 (Testing): 154/154, 100%, Done -- all 13 sprints green.
  - Epic 6 total 195 -> 202 in the Master Tracker (the 7 Dex chips moved in).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Master_Tracker.xlsx
+++ b/docs/DecisionOS_Master_Tracker.xlsx
@@ -589,7 +589,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -705,19 +704,19 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>72%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
@@ -807,11 +806,11 @@
         <v>117</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -936,19 +935,19 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>31</v>
+        <v>154</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>154</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">

</xml_diff>